<commit_message>
feat: verify rule CG0085 and add negative test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000260/negative/01/data/unit-test-coreid-CG0085-negative 1.xlsx
+++ b/rules/CORE-000260/negative/01/data/unit-test-coreid-CG0085-negative 1.xlsx
@@ -35,7 +35,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +46,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
         <bgColor rgb="00FFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -89,6 +95,9 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -532,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -564,6 +573,258 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AEPRESP</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AEPRESP</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>AEPRESP</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>8</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>AEPRESP</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>9</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>AEPRESP</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>AEPRESP</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>11</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>AEPRESP</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>12</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>AEPRESP</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>13</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>AEPRESP</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1564,7 @@
           <t>INJECTION SITE REACTION</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="O5" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1419,7 +1680,7 @@
           <t>SHOULDER PAIN</t>
         </is>
       </c>
-      <c r="O6" s="4" t="inlineStr">
+      <c r="O6" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1535,7 +1796,7 @@
           <t>FEELING ABNORMAL</t>
         </is>
       </c>
-      <c r="O7" s="4" t="inlineStr">
+      <c r="O7" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1651,7 +1912,7 @@
           <t>LIBIDO DECREASED</t>
         </is>
       </c>
-      <c r="O8" s="4" t="inlineStr">
+      <c r="O8" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1767,7 +2028,7 @@
           <t>LISTLESS</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr">
+      <c r="O9" s="6" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -1883,7 +2144,7 @@
           <t>INJECTION SITE REACTION</t>
         </is>
       </c>
-      <c r="O10" s="4" t="inlineStr">
+      <c r="O10" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1997,7 +2258,7 @@
           <t>INJECTION SITE REACTION</t>
         </is>
       </c>
-      <c r="O11" s="4" t="inlineStr">
+      <c r="O11" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2113,7 +2374,7 @@
           <t>INJECTION SITE REACTION</t>
         </is>
       </c>
-      <c r="O12" s="4" t="inlineStr">
+      <c r="O12" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2227,7 +2488,7 @@
           <t>INJECTION SITE REACTION</t>
         </is>
       </c>
-      <c r="O13" s="4" t="inlineStr">
+      <c r="O13" s="6" t="inlineStr">
         <is>
           <t>UNKNOWN</t>
         </is>

</xml_diff>